<commit_message>
added assessment strategy for MOO, fixed database error
</commit_message>
<xml_diff>
--- a/data/dynamic_systems.xlsx
+++ b/data/dynamic_systems.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mim26609\PycharmProjects\OptiGOBTimeSeries\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mim26609\workspace\claude\OptiGOBTimeSeries\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB311FE2-CAFE-4C9C-981C-C54C58301A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B178BB4-DDDF-4BFD-A96D-41ADCEF62AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cattle" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="61">
   <si>
     <t>Abatement</t>
   </si>
@@ -210,6 +210,18 @@
   </si>
   <si>
     <t>nh3</t>
+  </si>
+  <si>
+    <t>milk_yield</t>
+  </si>
+  <si>
+    <t>beef_carcass_yield</t>
+  </si>
+  <si>
+    <t>total_yield</t>
+  </si>
+  <si>
+    <t>raw_output</t>
   </si>
 </sst>
 </file>
@@ -608,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -1275,14 +1287,14 @@
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>18</v>
+      <c r="A12" t="s">
+        <v>57</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="3">
-        <v>54202500</v>
+        <v>54202.5</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
@@ -1291,831 +1303,1018 @@
         <v>0</v>
       </c>
       <c r="F12" s="3">
-        <v>62204760</v>
+        <v>62204.76</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
       </c>
       <c r="H12" s="3">
-        <v>70207020</v>
+        <v>70207.02</v>
       </c>
       <c r="I12" s="1">
         <v>0</v>
       </c>
       <c r="J12" s="3">
-        <v>54202500</v>
+        <v>54202.5</v>
       </c>
       <c r="K12" s="1">
         <v>0</v>
       </c>
       <c r="L12" s="3">
-        <v>62204760</v>
+        <v>62204.76</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
       </c>
       <c r="N12" s="3">
-        <v>70207020</v>
+        <v>70207.02</v>
       </c>
       <c r="O12" s="1">
         <v>0</v>
       </c>
       <c r="P12" s="3">
-        <v>54202500</v>
+        <v>54202.5</v>
       </c>
       <c r="Q12" s="1">
         <v>0</v>
       </c>
       <c r="R12" s="3">
-        <v>62204760</v>
+        <v>62204.76</v>
       </c>
       <c r="S12" s="1">
         <v>0</v>
       </c>
       <c r="T12" s="3">
-        <v>70207020</v>
+        <v>70207.02</v>
       </c>
       <c r="U12" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>20</v>
+      <c r="A13" t="s">
+        <v>58</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="D13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="E13" s="3">
         <v>0</v>
       </c>
       <c r="F13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="G13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="H13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="I13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="J13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="K13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="L13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="M13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="N13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="O13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="P13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="Q13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="R13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="S13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
       <c r="T13" s="3">
-        <v>2421607</v>
+        <v>2421.607</v>
       </c>
       <c r="U13" s="3">
-        <v>3008317</v>
+        <v>3008.317</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="3">
-        <v>56624107</v>
+        <f>0.035*C12</f>
+        <v>1897.0875000000001</v>
       </c>
       <c r="D14" s="3">
-        <v>3008317</v>
+        <f t="shared" ref="D14:U14" si="0">0.035*D12</f>
+        <v>0</v>
       </c>
       <c r="E14" s="3">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F14" s="3">
-        <v>64626367</v>
+        <f t="shared" si="0"/>
+        <v>2177.1666000000005</v>
       </c>
       <c r="G14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="H14" s="3">
-        <v>72628627</v>
+        <f t="shared" si="0"/>
+        <v>2457.2457000000004</v>
       </c>
       <c r="I14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="J14" s="3">
-        <v>56624107</v>
+        <f t="shared" si="0"/>
+        <v>1897.0875000000001</v>
       </c>
       <c r="K14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="L14" s="3">
-        <v>64626367</v>
+        <f t="shared" si="0"/>
+        <v>2177.1666000000005</v>
       </c>
       <c r="M14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="N14" s="3">
-        <v>72628627</v>
+        <f t="shared" si="0"/>
+        <v>2457.2457000000004</v>
       </c>
       <c r="O14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="P14" s="3">
-        <v>56624107</v>
+        <f t="shared" si="0"/>
+        <v>1897.0875000000001</v>
       </c>
       <c r="Q14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="R14" s="3">
-        <v>64626367</v>
+        <f t="shared" si="0"/>
+        <v>2177.1666000000005</v>
       </c>
       <c r="S14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="T14" s="3">
-        <v>72628627</v>
+        <f t="shared" si="0"/>
+        <v>2457.2457000000004</v>
       </c>
       <c r="U14" s="3">
-        <v>3008317</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C15" s="3">
-        <v>27439</v>
+        <f>0.23*C13</f>
+        <v>556.96960999999999</v>
       </c>
       <c r="D15" s="3">
-        <v>28177</v>
+        <f t="shared" ref="D15:U15" si="1">0.23*D13</f>
+        <v>691.91291000000001</v>
       </c>
       <c r="E15" s="3">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F15" s="3">
-        <v>27439</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="G15" s="3">
-        <v>28177</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="H15" s="3">
-        <v>25934</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="I15" s="3">
-        <v>26203</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="J15" s="3">
-        <v>27439</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="K15" s="3">
-        <v>28177</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="L15" s="3">
-        <v>27439</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="M15" s="3">
-        <v>28177</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="N15" s="3">
-        <v>25934</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="O15" s="3">
-        <v>26203</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="P15" s="3">
-        <v>27439</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="Q15" s="3">
-        <v>28177</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="R15" s="3">
-        <v>27439</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="S15" s="3">
-        <v>28177</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
       <c r="T15" s="3">
-        <v>25934</v>
+        <f t="shared" si="1"/>
+        <v>556.96960999999999</v>
       </c>
       <c r="U15" s="3">
-        <v>26203</v>
+        <f t="shared" si="1"/>
+        <v>691.91291000000001</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="2">
-        <v>1390.1</v>
-      </c>
-      <c r="D16" s="2">
-        <v>4784.5</v>
-      </c>
-      <c r="E16" s="2">
-        <v>0</v>
-      </c>
-      <c r="F16" s="2">
-        <v>1377.7</v>
-      </c>
-      <c r="G16" s="2">
-        <v>4585.1000000000004</v>
-      </c>
-      <c r="H16" s="2">
-        <v>1194.7</v>
-      </c>
-      <c r="I16" s="2">
-        <v>4385.7</v>
-      </c>
-      <c r="J16" s="2">
-        <v>1390.1</v>
-      </c>
-      <c r="K16" s="2">
-        <v>4784.5</v>
-      </c>
-      <c r="L16" s="2">
-        <v>1377.7</v>
-      </c>
-      <c r="M16" s="2">
-        <v>4585.1000000000004</v>
-      </c>
-      <c r="N16" s="2">
-        <v>1194.7</v>
-      </c>
-      <c r="O16" s="2">
-        <v>4385.7</v>
-      </c>
-      <c r="P16" s="2">
-        <v>1217.9000000000001</v>
-      </c>
-      <c r="Q16" s="2">
-        <v>3594.4</v>
-      </c>
-      <c r="R16" s="2">
-        <v>1215.2</v>
-      </c>
-      <c r="S16" s="2">
-        <v>3460.5</v>
-      </c>
-      <c r="T16" s="2">
-        <v>1060.9000000000001</v>
-      </c>
-      <c r="U16" s="2">
-        <v>3326.7</v>
+        <v>19</v>
+      </c>
+      <c r="C16" s="3">
+        <f>C12+C13</f>
+        <v>56624.107000000004</v>
+      </c>
+      <c r="D16" s="3">
+        <f t="shared" ref="D16:U16" si="2">D12+D13</f>
+        <v>3008.317</v>
+      </c>
+      <c r="E16" s="3">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F16" s="3">
+        <f t="shared" si="2"/>
+        <v>64626.366999999998</v>
+      </c>
+      <c r="G16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="H16" s="3">
+        <f t="shared" si="2"/>
+        <v>72628.627000000008</v>
+      </c>
+      <c r="I16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="J16" s="3">
+        <f t="shared" si="2"/>
+        <v>56624.107000000004</v>
+      </c>
+      <c r="K16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="L16" s="3">
+        <f t="shared" si="2"/>
+        <v>64626.366999999998</v>
+      </c>
+      <c r="M16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="N16" s="3">
+        <f t="shared" si="2"/>
+        <v>72628.627000000008</v>
+      </c>
+      <c r="O16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="P16" s="3">
+        <f t="shared" si="2"/>
+        <v>56624.107000000004</v>
+      </c>
+      <c r="Q16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="R16" s="3">
+        <f t="shared" si="2"/>
+        <v>64626.366999999998</v>
+      </c>
+      <c r="S16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
+      </c>
+      <c r="T16" s="3">
+        <f t="shared" si="2"/>
+        <v>72628.627000000008</v>
+      </c>
+      <c r="U16" s="3">
+        <f t="shared" si="2"/>
+        <v>3008.317</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C17" s="3">
-        <v>13895</v>
+        <v>27439</v>
       </c>
       <c r="D17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
       </c>
       <c r="F17" s="3">
-        <v>15721</v>
+        <v>27439</v>
       </c>
       <c r="G17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="H17" s="3">
-        <v>17546</v>
+        <v>25934</v>
       </c>
       <c r="I17" s="3">
-        <v>6228</v>
+        <v>26203</v>
       </c>
       <c r="J17" s="3">
-        <v>13895</v>
+        <v>27439</v>
       </c>
       <c r="K17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="L17" s="3">
-        <v>15721</v>
+        <v>27439</v>
       </c>
       <c r="M17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="N17" s="3">
-        <v>17546</v>
+        <v>25934</v>
       </c>
       <c r="O17" s="3">
-        <v>6228</v>
+        <v>26203</v>
       </c>
       <c r="P17" s="3">
-        <v>13895</v>
+        <v>27439</v>
       </c>
       <c r="Q17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="R17" s="3">
-        <v>15721</v>
+        <v>27439</v>
       </c>
       <c r="S17" s="3">
-        <v>6228</v>
+        <v>28177</v>
       </c>
       <c r="T17" s="3">
-        <v>17546</v>
+        <v>25934</v>
       </c>
       <c r="U17" s="3">
-        <v>6228</v>
+        <v>26203</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="1">
-        <v>966</v>
-      </c>
-      <c r="D18" s="3">
-        <v>1328</v>
-      </c>
-      <c r="E18" s="3">
-        <v>0</v>
-      </c>
-      <c r="F18" s="1">
-        <v>957</v>
-      </c>
-      <c r="G18" s="3">
-        <v>1273</v>
-      </c>
-      <c r="H18" s="1">
-        <v>951</v>
-      </c>
-      <c r="I18" s="3">
-        <v>1218</v>
-      </c>
-      <c r="J18" s="1">
-        <v>966</v>
-      </c>
-      <c r="K18" s="3">
-        <v>1328</v>
-      </c>
-      <c r="L18" s="1">
-        <v>957</v>
-      </c>
-      <c r="M18" s="3">
-        <v>1273</v>
-      </c>
-      <c r="N18" s="1">
-        <v>951</v>
-      </c>
-      <c r="O18" s="3">
-        <v>1218</v>
-      </c>
-      <c r="P18" s="1">
-        <v>846</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>998</v>
-      </c>
-      <c r="R18" s="1">
-        <v>846</v>
-      </c>
-      <c r="S18" s="1">
-        <v>961</v>
-      </c>
-      <c r="T18" s="1">
-        <v>846</v>
-      </c>
-      <c r="U18" s="1">
-        <v>924</v>
+        <v>16</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1390.1</v>
+      </c>
+      <c r="D18" s="2">
+        <v>4784.5</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <v>1377.7</v>
+      </c>
+      <c r="G18" s="2">
+        <v>4585.1000000000004</v>
+      </c>
+      <c r="H18" s="2">
+        <v>1194.7</v>
+      </c>
+      <c r="I18" s="2">
+        <v>4385.7</v>
+      </c>
+      <c r="J18" s="2">
+        <v>1390.1</v>
+      </c>
+      <c r="K18" s="2">
+        <v>4784.5</v>
+      </c>
+      <c r="L18" s="2">
+        <v>1377.7</v>
+      </c>
+      <c r="M18" s="2">
+        <v>4585.1000000000004</v>
+      </c>
+      <c r="N18" s="2">
+        <v>1194.7</v>
+      </c>
+      <c r="O18" s="2">
+        <v>4385.7</v>
+      </c>
+      <c r="P18" s="2">
+        <v>1217.9000000000001</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>3594.4</v>
+      </c>
+      <c r="R18" s="2">
+        <v>1215.2</v>
+      </c>
+      <c r="S18" s="2">
+        <v>3460.5</v>
+      </c>
+      <c r="T18" s="2">
+        <v>1060.9000000000001</v>
+      </c>
+      <c r="U18" s="2">
+        <v>3326.7</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="1">
-        <v>111</v>
-      </c>
-      <c r="D19" s="1">
-        <v>153</v>
-      </c>
-      <c r="E19" s="1">
-        <v>0</v>
-      </c>
-      <c r="F19" s="1">
-        <v>110</v>
-      </c>
-      <c r="G19" s="1">
-        <v>147</v>
-      </c>
-      <c r="H19" s="1">
-        <v>110</v>
-      </c>
-      <c r="I19" s="1">
-        <v>140</v>
-      </c>
-      <c r="J19" s="1">
-        <v>111</v>
-      </c>
-      <c r="K19" s="1">
-        <v>153</v>
-      </c>
-      <c r="L19" s="1">
-        <v>110</v>
-      </c>
-      <c r="M19" s="1">
-        <v>147</v>
-      </c>
-      <c r="N19" s="1">
-        <v>110</v>
-      </c>
-      <c r="O19" s="1">
-        <v>140</v>
-      </c>
-      <c r="P19" s="1">
-        <v>97</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>115</v>
-      </c>
-      <c r="R19" s="1">
-        <v>97</v>
-      </c>
-      <c r="S19" s="1">
-        <v>111</v>
-      </c>
-      <c r="T19" s="1">
-        <v>97</v>
-      </c>
-      <c r="U19" s="1">
-        <v>106</v>
+      <c r="C19" s="3">
+        <v>13895</v>
+      </c>
+      <c r="D19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>15721</v>
+      </c>
+      <c r="G19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="H19" s="3">
+        <v>17546</v>
+      </c>
+      <c r="I19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="J19" s="3">
+        <v>13895</v>
+      </c>
+      <c r="K19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="L19" s="3">
+        <v>15721</v>
+      </c>
+      <c r="M19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="N19" s="3">
+        <v>17546</v>
+      </c>
+      <c r="O19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="P19" s="3">
+        <v>13895</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="R19" s="3">
+        <v>15721</v>
+      </c>
+      <c r="S19" s="3">
+        <v>6228</v>
+      </c>
+      <c r="T19" s="3">
+        <v>17546</v>
+      </c>
+      <c r="U19" s="3">
+        <v>6228</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="1">
-        <v>362</v>
-      </c>
-      <c r="D20" s="1">
-        <v>498</v>
-      </c>
-      <c r="E20" s="1">
+        <v>966</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1328</v>
+      </c>
+      <c r="E20" s="3">
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>359</v>
-      </c>
-      <c r="G20" s="1">
-        <v>477</v>
+        <v>957</v>
+      </c>
+      <c r="G20" s="3">
+        <v>1273</v>
       </c>
       <c r="H20" s="1">
-        <v>356</v>
-      </c>
-      <c r="I20" s="1">
-        <v>456</v>
+        <v>951</v>
+      </c>
+      <c r="I20" s="3">
+        <v>1218</v>
       </c>
       <c r="J20" s="1">
-        <v>362</v>
-      </c>
-      <c r="K20" s="1">
-        <v>498</v>
+        <v>966</v>
+      </c>
+      <c r="K20" s="3">
+        <v>1328</v>
       </c>
       <c r="L20" s="1">
-        <v>359</v>
-      </c>
-      <c r="M20" s="1">
-        <v>477</v>
+        <v>957</v>
+      </c>
+      <c r="M20" s="3">
+        <v>1273</v>
       </c>
       <c r="N20" s="1">
-        <v>356</v>
-      </c>
-      <c r="O20" s="1">
-        <v>456</v>
+        <v>951</v>
+      </c>
+      <c r="O20" s="3">
+        <v>1218</v>
       </c>
       <c r="P20" s="1">
-        <v>317</v>
+        <v>846</v>
       </c>
       <c r="Q20" s="1">
-        <v>374</v>
+        <v>998</v>
       </c>
       <c r="R20" s="1">
-        <v>317</v>
+        <v>846</v>
       </c>
       <c r="S20" s="1">
-        <v>360</v>
+        <v>961</v>
       </c>
       <c r="T20" s="1">
-        <v>317</v>
+        <v>846</v>
       </c>
       <c r="U20" s="1">
-        <v>346</v>
+        <v>924</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C21" s="1">
-        <v>0.37</v>
+        <v>111</v>
       </c>
       <c r="D21" s="1">
-        <v>0.41</v>
+        <v>153</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>0.37</v>
+        <v>110</v>
       </c>
       <c r="G21" s="1">
-        <v>0.41</v>
+        <v>147</v>
       </c>
       <c r="H21" s="1">
-        <v>0.37</v>
+        <v>110</v>
       </c>
       <c r="I21" s="1">
-        <v>0.41</v>
+        <v>140</v>
       </c>
       <c r="J21" s="1">
-        <v>0.37</v>
+        <v>111</v>
       </c>
       <c r="K21" s="1">
-        <v>0.41</v>
+        <v>153</v>
       </c>
       <c r="L21" s="1">
-        <v>0.37</v>
+        <v>110</v>
       </c>
       <c r="M21" s="1">
-        <v>0.41</v>
+        <v>147</v>
       </c>
       <c r="N21" s="1">
-        <v>0.37</v>
+        <v>110</v>
       </c>
       <c r="O21" s="1">
-        <v>0.41</v>
+        <v>140</v>
       </c>
       <c r="P21" s="1">
-        <v>0.38</v>
+        <v>97</v>
       </c>
       <c r="Q21" s="1">
-        <v>0.38</v>
+        <v>115</v>
       </c>
       <c r="R21" s="1">
-        <v>0.38</v>
+        <v>97</v>
       </c>
       <c r="S21" s="1">
-        <v>0.38</v>
+        <v>111</v>
       </c>
       <c r="T21" s="1">
-        <v>0.38</v>
+        <v>97</v>
       </c>
       <c r="U21" s="1">
-        <v>0.38</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C22" s="1">
-        <v>0.39</v>
+        <v>362</v>
       </c>
       <c r="D22" s="1">
-        <v>0.46</v>
+        <v>498</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>0.39</v>
+        <v>359</v>
       </c>
       <c r="G22" s="1">
-        <v>0.46</v>
+        <v>477</v>
       </c>
       <c r="H22" s="1">
-        <v>0.39</v>
+        <v>356</v>
       </c>
       <c r="I22" s="1">
-        <v>0.46</v>
+        <v>456</v>
       </c>
       <c r="J22" s="1">
-        <v>0.39</v>
+        <v>362</v>
       </c>
       <c r="K22" s="1">
-        <v>0.46</v>
+        <v>498</v>
       </c>
       <c r="L22" s="1">
-        <v>0.39</v>
+        <v>359</v>
       </c>
       <c r="M22" s="1">
-        <v>0.46</v>
+        <v>477</v>
       </c>
       <c r="N22" s="1">
-        <v>0.39</v>
+        <v>356</v>
       </c>
       <c r="O22" s="1">
-        <v>0.46</v>
+        <v>456</v>
       </c>
       <c r="P22" s="1">
-        <v>0.39</v>
+        <v>317</v>
       </c>
       <c r="Q22" s="1">
-        <v>0.38</v>
+        <v>374</v>
       </c>
       <c r="R22" s="1">
-        <v>0.39</v>
+        <v>317</v>
       </c>
       <c r="S22" s="1">
-        <v>0.38</v>
+        <v>360</v>
       </c>
       <c r="T22" s="1">
-        <v>0.39</v>
+        <v>317</v>
       </c>
       <c r="U22" s="1">
-        <v>0.38</v>
+        <v>346</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="D23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="G23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="H23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="I23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="J23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="K23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="L23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="M23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="N23" s="1">
-        <v>0.02</v>
+        <v>0.37</v>
       </c>
       <c r="O23" s="1">
-        <v>0.02</v>
+        <v>0.41</v>
       </c>
       <c r="P23" s="1">
-        <v>0.03</v>
+        <v>0.38</v>
       </c>
       <c r="Q23" s="1">
-        <v>0.02</v>
+        <v>0.38</v>
       </c>
       <c r="R23" s="1">
-        <v>0.03</v>
+        <v>0.38</v>
       </c>
       <c r="S23" s="1">
-        <v>0.02</v>
+        <v>0.38</v>
       </c>
       <c r="T23" s="1">
-        <v>0.03</v>
+        <v>0.38</v>
       </c>
       <c r="U23" s="1">
-        <v>0.02</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="H24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="I24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="K24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="L24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="M24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="N24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="O24" s="1">
+        <v>0.46</v>
+      </c>
+      <c r="P24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="R24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="S24" s="1">
+        <v>0.38</v>
+      </c>
+      <c r="T24" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="U24" s="1">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="I25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="J25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="K25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="L25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="M25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="N25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="O25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="P25" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="Q25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="R25" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="S25" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="T25" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="U25" s="1">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C26" s="3">
         <v>5918</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D26" s="3">
         <v>2219</v>
       </c>
-      <c r="E24" s="3">
-        <v>0</v>
-      </c>
-      <c r="F24" s="3">
+      <c r="E26" s="3">
+        <v>0</v>
+      </c>
+      <c r="F26" s="3">
         <v>6300</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G26" s="3">
         <v>2242</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H26" s="3">
         <v>6681</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I26" s="3">
         <v>2265</v>
       </c>
-      <c r="J24" s="3">
+      <c r="J26" s="3">
         <v>5918</v>
       </c>
-      <c r="K24" s="3">
+      <c r="K26" s="3">
         <v>2219</v>
       </c>
-      <c r="L24" s="3">
+      <c r="L26" s="3">
         <v>6300</v>
       </c>
-      <c r="M24" s="3">
+      <c r="M26" s="3">
         <v>2242</v>
       </c>
-      <c r="N24" s="3">
+      <c r="N26" s="3">
         <v>6681</v>
       </c>
-      <c r="O24" s="3">
+      <c r="O26" s="3">
         <v>2265</v>
       </c>
-      <c r="P24" s="3">
+      <c r="P26" s="3">
         <v>5918</v>
       </c>
-      <c r="Q24" s="3">
+      <c r="Q26" s="3">
         <v>2219</v>
       </c>
-      <c r="R24" s="3">
+      <c r="R26" s="3">
         <v>6300</v>
       </c>
-      <c r="S24" s="3">
+      <c r="S26" s="3">
         <v>2242</v>
       </c>
-      <c r="T24" s="3">
+      <c r="T26" s="3">
         <v>6681</v>
       </c>
-      <c r="U24" s="3">
+      <c r="U26" s="3">
         <v>2265</v>
       </c>
     </row>
@@ -2126,7 +2325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{068914BF-AE90-4BE8-894C-61EC99CA55D7}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -2517,7 +2716,7 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>19</v>
@@ -2564,110 +2763,123 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="2">
-        <v>55453.7</v>
+        <f>C10*0.25</f>
+        <v>13863.424999999999</v>
       </c>
       <c r="D11" s="2">
-        <v>30628</v>
+        <f>D10*0.27</f>
+        <v>8269.5600000000013</v>
       </c>
       <c r="E11" s="2">
-        <v>176358.5</v>
+        <f t="shared" ref="E11:O11" si="0">E10*0.25</f>
+        <v>67830.2</v>
       </c>
       <c r="F11" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G11" s="2">
-        <v>6891.5</v>
+        <f t="shared" si="0"/>
+        <v>1722.875</v>
       </c>
       <c r="H11" s="2">
-        <v>55453.7</v>
+        <f t="shared" si="0"/>
+        <v>13863.424999999999</v>
       </c>
       <c r="I11" s="2">
-        <v>30628</v>
+        <f>I10*0.27</f>
+        <v>8269.5600000000013</v>
       </c>
       <c r="J11" s="2">
-        <v>193112.6</v>
+        <f t="shared" si="0"/>
+        <v>74274.074999999997</v>
       </c>
       <c r="K11" s="2">
-        <v>6891.5</v>
+        <f t="shared" si="0"/>
+        <v>1722.875</v>
       </c>
       <c r="L11" s="2">
-        <v>55453.7</v>
+        <f t="shared" si="0"/>
+        <v>13863.424999999999</v>
       </c>
       <c r="M11" s="2">
-        <v>30628</v>
+        <f>M10*0.27</f>
+        <v>8269.5600000000013</v>
       </c>
       <c r="N11" s="2">
-        <v>209866.6</v>
+        <f t="shared" si="0"/>
+        <v>80717.925000000003</v>
       </c>
       <c r="O11" s="2">
-        <v>6891.5</v>
+        <f t="shared" si="0"/>
+        <v>1722.875</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="1">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2">
+        <v>55453.7</v>
+      </c>
+      <c r="D12" s="2">
+        <v>30628</v>
+      </c>
+      <c r="E12" s="2">
+        <v>176358.5</v>
+      </c>
+      <c r="F12" s="2">
         <v>0</v>
       </c>
       <c r="G12" s="2">
-        <v>276006.8</v>
-      </c>
-      <c r="H12" s="1">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>0</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0</v>
+        <v>6891.5</v>
+      </c>
+      <c r="H12" s="2">
+        <v>55453.7</v>
+      </c>
+      <c r="I12" s="2">
+        <v>30628</v>
+      </c>
+      <c r="J12" s="2">
+        <v>193112.6</v>
       </c>
       <c r="K12" s="2">
-        <v>276006.8</v>
-      </c>
-      <c r="L12" s="1">
-        <v>0</v>
-      </c>
-      <c r="M12" s="1">
-        <v>0</v>
-      </c>
-      <c r="N12" s="1">
-        <v>0</v>
+        <v>6891.5</v>
+      </c>
+      <c r="L12" s="2">
+        <v>55453.7</v>
+      </c>
+      <c r="M12" s="2">
+        <v>30628</v>
+      </c>
+      <c r="N12" s="2">
+        <v>209866.6</v>
       </c>
       <c r="O12" s="2">
-        <v>198549</v>
+        <v>6891.5</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="2">
-        <v>1322672.5</v>
-      </c>
-      <c r="D13" s="2">
-        <v>513073.8</v>
+        <v>16</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -2676,83 +2888,83 @@
         <v>0</v>
       </c>
       <c r="G13" s="2">
-        <v>299336.40000000002</v>
-      </c>
-      <c r="H13" s="2">
-        <v>1322672.5</v>
-      </c>
-      <c r="I13" s="2">
-        <v>513073.8</v>
+        <v>276006.8</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
       </c>
       <c r="J13" s="1">
         <v>0</v>
       </c>
       <c r="K13" s="2">
-        <v>299336.40000000002</v>
-      </c>
-      <c r="L13" s="2">
-        <v>1322672.5</v>
-      </c>
-      <c r="M13" s="2">
-        <v>513073.8</v>
+        <v>276006.8</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="2">
-        <v>299336.40000000002</v>
+        <v>198549</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="1">
-        <v>0</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2">
-        <v>42368.9</v>
-      </c>
-      <c r="F14" s="2">
+      <c r="C14" s="2">
+        <v>1322672.5</v>
+      </c>
+      <c r="D14" s="2">
+        <v>513073.8</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="2">
-        <v>76626</v>
-      </c>
-      <c r="H14" s="1">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2">
-        <v>42368.9</v>
+        <v>299336.40000000002</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1322672.5</v>
+      </c>
+      <c r="I14" s="2">
+        <v>513073.8</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0</v>
       </c>
       <c r="K14" s="2">
-        <v>76626</v>
-      </c>
-      <c r="L14" s="1">
-        <v>0</v>
-      </c>
-      <c r="M14" s="1">
-        <v>0</v>
-      </c>
-      <c r="N14" s="2">
-        <v>42368.9</v>
+        <v>299336.40000000002</v>
+      </c>
+      <c r="L14" s="2">
+        <v>1322672.5</v>
+      </c>
+      <c r="M14" s="2">
+        <v>513073.8</v>
+      </c>
+      <c r="N14" s="1">
+        <v>0</v>
       </c>
       <c r="O14" s="2">
-        <v>55121.9</v>
+        <v>299336.40000000002</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>19</v>
@@ -2764,13 +2976,13 @@
         <v>0</v>
       </c>
       <c r="E15" s="2">
-        <v>11050.2</v>
+        <v>42368.9</v>
       </c>
       <c r="F15" s="2">
         <v>0</v>
       </c>
       <c r="G15" s="2">
-        <v>8824.7000000000007</v>
+        <v>76626</v>
       </c>
       <c r="H15" s="1">
         <v>0</v>
@@ -2779,10 +2991,10 @@
         <v>0</v>
       </c>
       <c r="J15" s="2">
-        <v>11050.2</v>
+        <v>42368.9</v>
       </c>
       <c r="K15" s="2">
-        <v>8824.7000000000007</v>
+        <v>76626</v>
       </c>
       <c r="L15" s="1">
         <v>0</v>
@@ -2791,15 +3003,15 @@
         <v>0</v>
       </c>
       <c r="N15" s="2">
-        <v>11050.2</v>
+        <v>42368.9</v>
       </c>
       <c r="O15" s="2">
-        <v>6348.2</v>
+        <v>55121.9</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>19</v>
@@ -2811,13 +3023,13 @@
         <v>0</v>
       </c>
       <c r="E16" s="2">
-        <v>35765.5</v>
+        <v>11050.2</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
       </c>
       <c r="G16" s="2">
-        <v>28722.799999999999</v>
+        <v>8824.7000000000007</v>
       </c>
       <c r="H16" s="1">
         <v>0</v>
@@ -2826,10 +3038,10 @@
         <v>0</v>
       </c>
       <c r="J16" s="2">
-        <v>35765.5</v>
+        <v>11050.2</v>
       </c>
       <c r="K16" s="2">
-        <v>28722.799999999999</v>
+        <v>8824.7000000000007</v>
       </c>
       <c r="L16" s="1">
         <v>0</v>
@@ -2838,197 +3050,244 @@
         <v>0</v>
       </c>
       <c r="N16" s="2">
-        <v>35765.5</v>
+        <v>11050.2</v>
       </c>
       <c r="O16" s="2">
-        <v>20662.099999999999</v>
+        <v>6348.2</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C17" s="1">
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
       <c r="D17" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="E17" s="1">
-        <v>2.8</v>
-      </c>
-      <c r="F17" s="1">
-        <v>0</v>
-      </c>
-      <c r="G17" s="1">
-        <v>5.6</v>
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>35765.5</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>28722.799999999999</v>
       </c>
       <c r="H17" s="1">
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
       <c r="I17" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="J17" s="1">
-        <v>2.8</v>
-      </c>
-      <c r="K17" s="1">
-        <v>5.6</v>
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>35765.5</v>
+      </c>
+      <c r="K17" s="2">
+        <v>28722.799999999999</v>
       </c>
       <c r="L17" s="1">
-        <v>1.1000000000000001</v>
+        <v>0</v>
       </c>
       <c r="M17" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="N17" s="1">
-        <v>2.8</v>
-      </c>
-      <c r="O17" s="1">
-        <v>3.8</v>
+        <v>0</v>
+      </c>
+      <c r="N17" s="2">
+        <v>35765.5</v>
+      </c>
+      <c r="O17" s="2">
+        <v>20662.099999999999</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="1">
-        <v>1.3</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D18" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="E18" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="H18" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="E18" s="1">
-        <v>12.8</v>
-      </c>
-      <c r="F18" s="1">
-        <v>0</v>
-      </c>
-      <c r="G18" s="1">
-        <v>24.6</v>
-      </c>
-      <c r="H18" s="1">
-        <v>1.3</v>
-      </c>
       <c r="I18" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="J18" s="1">
+        <v>2.8</v>
+      </c>
+      <c r="K18" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="L18" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J18" s="1">
-        <v>12.8</v>
-      </c>
-      <c r="K18" s="1">
-        <v>24.6</v>
-      </c>
-      <c r="L18" s="1">
-        <v>1.3</v>
-      </c>
       <c r="M18" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="N18" s="1">
-        <v>12.8</v>
+        <v>2.8</v>
       </c>
       <c r="O18" s="1">
-        <v>18.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="1">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="D19" s="1">
-        <v>0.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E19" s="1">
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
       </c>
       <c r="G19" s="1">
-        <v>2.6</v>
+        <v>24.6</v>
       </c>
       <c r="H19" s="1">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="I19" s="1">
-        <v>0.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="J19" s="1">
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="K19" s="1">
-        <v>2.6</v>
+        <v>24.6</v>
       </c>
       <c r="L19" s="1">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="M19" s="1">
-        <v>0.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="N19" s="1">
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="O19" s="1">
-        <v>1.8</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>2.6</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C21" s="2">
         <v>205096.1</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D21" s="2">
         <v>233019</v>
       </c>
-      <c r="E20" s="1">
-        <v>0</v>
-      </c>
-      <c r="F20" s="1">
-        <v>0</v>
-      </c>
-      <c r="G20" s="1">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
         <v>205096.1</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I21" s="2">
         <v>233019</v>
       </c>
-      <c r="J20" s="1">
-        <v>0</v>
-      </c>
-      <c r="K20" s="1">
-        <v>0</v>
-      </c>
-      <c r="L20" s="2">
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2">
         <v>205096.1</v>
       </c>
-      <c r="M20" s="2">
+      <c r="M21" s="2">
         <v>233019</v>
       </c>
-      <c r="N20" s="1">
-        <v>0</v>
-      </c>
-      <c r="O20" s="1">
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>